<commit_message>
Corrige cota de solera del sótano a -2,20 m según esquema vertical del DWG
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WUzF3Zu1dxVH3qtS5tHUab
</commit_message>
<xml_diff>
--- a/Fluidos_ET48/ET48_AF_ACS_calculo_v1.xlsx
+++ b/Fluidos_ET48/ET48_AF_ACS_calculo_v1.xlsx
@@ -771,8 +771,8 @@
           <t>Cota solera sótano</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
-        <v>-3</v>
+      <c r="B16" s="5" t="n">
+        <v>-2.2</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
@@ -781,7 +781,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>HIPÓTESIS: no acotada en el DWG; medir en sección</t>
+          <t>Esquema vertical DWG: cota 2,198 m bajo calzada 0,00 (rampa 12 m al 18 % = 2,16 m)</t>
         </is>
       </c>
     </row>

</xml_diff>